<commit_message>
Kestrel part 1: correct the generator (negative bills) and cross-check the key against the files
The first Noesi run showed the key's bill and payment totals 17,136.00 and
15,886.00 below the files. Cause: the generator produced negative bills
(an Alder & Finch fee bill, and office bills when the split bills and tool
rental exceeded the office budget). Fees are now spread around the fixed
June bill, the split bills sit under a 2,500 approval limit, tool rental
posts to freight, every bill and payment is asserted positive, and the key's
totals are re-read from the written files and asserted equal. Corrected
before any finding is recorded; the frozen part-0 files and key are
unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/case-studies/kestrel-valley-cycle/data/quickbooks/Bill_Payment_List.xlsx
+++ b/case-studies/kestrel-valley-cycle/data/quickbooks/Bill_Payment_List.xlsx
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="E9" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="10">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="E12" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="13">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="E15" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="16">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="E18" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="19">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E21" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="22">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="E24" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="25">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="E27" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="28">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="E30" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="31">
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="E33" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="34">
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="E36" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="37">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="E39" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="40">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="E42" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="43">
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="E43" s="1" t="n">
-        <v>-4950</v>
+        <v>-2450</v>
       </c>
     </row>
     <row r="44">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="E44" s="1" t="n">
-        <v>-4975</v>
+        <v>-2475</v>
       </c>
     </row>
     <row r="45">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="E45" s="1" t="n">
-        <v>-4900</v>
+        <v>-2400</v>
       </c>
     </row>
     <row r="46">
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="E48" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="49">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="E51" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="52">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="E54" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="55">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="E57" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="58">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="E60" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="61">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E63" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="64">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="E66" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="67">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="E69" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="70">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="E72" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="73">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="E75" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="76">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="E78" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="79">
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="E81" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="82">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E84" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="85">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="E87" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="88">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="E90" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="91">
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="E94" s="1" t="n">
-        <v>-722.09</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="95">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="E97" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.67</v>
       </c>
     </row>
     <row r="98">
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="E100" s="1" t="n">
-        <v>-8124.91</v>
+        <v>-7866.58</v>
       </c>
     </row>
     <row r="101">
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="E103" s="1" t="n">
-        <v>-722.1</v>
+        <v>-241.5</v>
       </c>
     </row>
     <row r="104">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="E106" s="1" t="n">
-        <v>-133449.16</v>
+        <v>-133425.69</v>
       </c>
     </row>
     <row r="107">
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="E109" s="1" t="n">
-        <v>-8124.9</v>
+        <v>-7866.57</v>
       </c>
     </row>
     <row r="110">
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="E122" s="1" t="n">
-        <v>-3300926.78</v>
+        <v>-3285040.78</v>
       </c>
     </row>
     <row r="123"/>

</xml_diff>

<commit_message>
Kestrel D10: sequential check numbers, one planted gap, a vendor named after an employee
- Checks renumbered 4267-4433 without a break (June 4411-4426; the key's
  4421, 4425, 4429, 4433 kept; four routine July checks added). One planted
  gap: checks 4422-4424 are not in QuickBooks.
- Owen Pike Hauling, a vendor named after employee E08 (5,925.00 of
  freight, moved from Velo's budget; trial balances unchanged). By name:
  the Vendor Contact List carries no bank account.
- Key lines (answer_key_part3 forensic, answer_key_payables
  vendor_employee_match), re-derived from the files in check_key.py
  (21/21), and five finish-line lines, all matching: 167/169, 0
  unexplained.
- Learn key and records regenerated; records select Moraine's payments by
  date, not by the old check numbers. The Journal size test reads the key.

529 tests pass; check-lessons passes. Not reviewed by a second agent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/case-studies/kestrel-valley-cycle/data/quickbooks/Bill_Payment_List.xlsx
+++ b/case-studies/kestrel-valley-cycle/data/quickbooks/Bill_Payment_List.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4002</t>
+          <t>4268</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4003</t>
+          <t>4269</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>4004</t>
+          <t>4270</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4005</t>
+          <t>4271</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4006</t>
+          <t>4272</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4007</t>
+          <t>4273</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="E12" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +598,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4008</t>
+          <t>4274</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4009</t>
+          <t>4275</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4010</t>
+          <t>4276</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="E15" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="16">
@@ -658,7 +658,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>4015</t>
+          <t>4281</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>4282</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4017</t>
+          <t>4283</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4018</t>
+          <t>4284</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>4019</t>
+          <t>4285</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>4286</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E21" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="22">
@@ -778,7 +778,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4021</t>
+          <t>4287</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4022</t>
+          <t>4288</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4023</t>
+          <t>4289</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="E24" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="25">
@@ -838,7 +838,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4027</t>
+          <t>4293</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>4294</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4029</t>
+          <t>4295</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4030</t>
+          <t>4296</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4031</t>
+          <t>4297</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4032</t>
+          <t>4298</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="E30" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="31">
@@ -958,7 +958,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>4033</t>
+          <t>4299</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4034</t>
+          <t>4300</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4035</t>
+          <t>4301</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1007,27 +1007,27 @@
         </is>
       </c>
       <c r="E33" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>10/20/2025</t>
+          <t>09/23/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>4041</t>
+          <t>4303</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Owen Pike Hauling</t>
         </is>
       </c>
       <c r="E34" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-1850</v>
       </c>
     </row>
     <row r="35">
@@ -1038,16 +1038,16 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>4042</t>
+          <t>4308</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E35" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="36">
@@ -1058,16 +1058,16 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>4043</t>
+          <t>4309</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E36" s="1" t="n">
-        <v>-241.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="37">
@@ -1078,16 +1078,16 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>4044</t>
+          <t>4310</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E37" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="38">
@@ -1098,16 +1098,16 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>4045</t>
+          <t>4311</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E38" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="39">
@@ -1118,16 +1118,16 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>4046</t>
+          <t>4312</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E39" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="40">
@@ -1138,16 +1138,16 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>4047</t>
+          <t>4313</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E40" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="41">
@@ -1158,16 +1158,16 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>4048</t>
+          <t>4314</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E41" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="42">
@@ -1178,36 +1178,36 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>4049</t>
+          <t>4315</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E42" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/14/2025</t>
+          <t>10/20/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>4053</t>
+          <t>4316</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Hyalite Fabrication</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E43" s="1" t="n">
-        <v>-2450</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="44">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>4054</t>
+          <t>4320</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="E44" s="1" t="n">
-        <v>-2475</v>
+        <v>-2450</v>
       </c>
     </row>
     <row r="45">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>4055</t>
+          <t>4321</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1247,27 +1247,27 @@
         </is>
       </c>
       <c r="E45" s="1" t="n">
-        <v>-2400</v>
+        <v>-2475</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/18/2025</t>
+          <t>11/14/2025</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>4056</t>
+          <t>4322</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Hyalite Fabrication</t>
         </is>
       </c>
       <c r="E46" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-2400</v>
       </c>
     </row>
     <row r="47">
@@ -1278,16 +1278,16 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>4057</t>
+          <t>4323</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E47" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="48">
@@ -1298,16 +1298,16 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>4058</t>
+          <t>4324</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E48" s="1" t="n">
-        <v>-241.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="49">
@@ -1318,16 +1318,16 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>4059</t>
+          <t>4325</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E49" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="50">
@@ -1338,16 +1338,16 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>4060</t>
+          <t>4326</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E50" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="51">
@@ -1358,16 +1358,16 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>4061</t>
+          <t>4327</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E51" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="52">
@@ -1378,16 +1378,16 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>4062</t>
+          <t>4328</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E52" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="53">
@@ -1398,16 +1398,16 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4063</t>
+          <t>4329</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E53" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="54">
@@ -1418,36 +1418,36 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>4064</t>
+          <t>4330</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E54" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>12/18/2025</t>
+          <t>11/18/2025</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>4068</t>
+          <t>4331</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E55" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="56">
@@ -1458,16 +1458,16 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>4069</t>
+          <t>4335</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E56" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="57">
@@ -1478,16 +1478,16 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>4070</t>
+          <t>4336</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E57" s="1" t="n">
-        <v>-241.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="58">
@@ -1498,16 +1498,16 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>4071</t>
+          <t>4337</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E58" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="59">
@@ -1518,16 +1518,16 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>4072</t>
+          <t>4338</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E59" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="60">
@@ -1538,16 +1538,16 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>4073</t>
+          <t>4339</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E60" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="61">
@@ -1558,16 +1558,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>4074</t>
+          <t>4340</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E61" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="62">
@@ -1578,16 +1578,16 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>4075</t>
+          <t>4341</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E62" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="63">
@@ -1598,36 +1598,36 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>4076</t>
+          <t>4342</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E63" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>01/19/2026</t>
+          <t>12/18/2025</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>4081</t>
+          <t>4343</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E64" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="65">
@@ -1638,16 +1638,16 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4348</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E65" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="66">
@@ -1658,16 +1658,16 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>4083</t>
+          <t>4349</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E66" s="1" t="n">
-        <v>-241.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="67">
@@ -1678,16 +1678,16 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4084</t>
+          <t>4350</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E67" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="68">
@@ -1698,16 +1698,16 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>4085</t>
+          <t>4351</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E68" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="69">
@@ -1718,16 +1718,16 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>4086</t>
+          <t>4352</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E69" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="70">
@@ -1738,16 +1738,16 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>4087</t>
+          <t>4353</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E70" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="71">
@@ -1758,16 +1758,16 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4088</t>
+          <t>4354</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E71" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="72">
@@ -1778,56 +1778,56 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>4089</t>
+          <t>4355</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E72" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>02/18/2026</t>
+          <t>01/19/2026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>4093</t>
+          <t>4356</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E73" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>02/18/2026</t>
+          <t>01/27/2026</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>4094</t>
+          <t>4359</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Owen Pike Hauling</t>
         </is>
       </c>
       <c r="E74" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-2100</v>
       </c>
     </row>
     <row r="75">
@@ -1838,16 +1838,16 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>4095</t>
+          <t>4361</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E75" s="1" t="n">
-        <v>-241.55</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="76">
@@ -1858,16 +1858,16 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>4096</t>
+          <t>4362</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E76" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="77">
@@ -1878,16 +1878,16 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>4097</t>
+          <t>4363</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E77" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="78">
@@ -1898,16 +1898,16 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>4098</t>
+          <t>4364</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E78" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="79">
@@ -1918,16 +1918,16 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>4099</t>
+          <t>4365</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E79" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="80">
@@ -1938,16 +1938,16 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>4366</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E80" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="81">
@@ -1958,56 +1958,56 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>4101</t>
+          <t>4367</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E81" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>03/18/2026</t>
+          <t>02/18/2026</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>4105</t>
+          <t>4368</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E82" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>03/18/2026</t>
+          <t>02/18/2026</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>4106</t>
+          <t>4369</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E83" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="84">
@@ -2018,16 +2018,16 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>4107</t>
+          <t>4373</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E84" s="1" t="n">
-        <v>-241.55</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="85">
@@ -2038,16 +2038,16 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>4108</t>
+          <t>4374</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E85" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="86">
@@ -2058,16 +2058,16 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>4109</t>
+          <t>4375</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E86" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="87">
@@ -2078,16 +2078,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>4110</t>
+          <t>4376</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E87" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="88">
@@ -2098,16 +2098,16 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>4111</t>
+          <t>4377</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E88" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="89">
@@ -2118,16 +2118,16 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>4112</t>
+          <t>4378</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E89" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="90">
@@ -2138,76 +2138,76 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>4113</t>
+          <t>4379</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E90" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>04/02/2026</t>
+          <t>03/18/2026</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>4117</t>
+          <t>4380</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components, Inc.</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E91" s="1" t="n">
-        <v>-18432.5</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>04/20/2026</t>
+          <t>03/18/2026</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>4119</t>
+          <t>4381</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E92" s="1" t="n">
-        <v>-1134.09</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>04/20/2026</t>
+          <t>04/02/2026</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>4385</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Moraine Cycle Components, Inc.</t>
         </is>
       </c>
       <c r="E93" s="1" t="n">
-        <v>-2045.45</v>
+        <v>-18432.5</v>
       </c>
     </row>
     <row r="94">
@@ -2218,16 +2218,16 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>4121</t>
+          <t>4387</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E94" s="1" t="n">
-        <v>-241.55</v>
+        <v>-1134.09</v>
       </c>
     </row>
     <row r="95">
@@ -2238,16 +2238,16 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>4122</t>
+          <t>4388</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E95" s="1" t="n">
-        <v>-7954.55</v>
+        <v>-2045.45</v>
       </c>
     </row>
     <row r="96">
@@ -2258,16 +2258,16 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>4123</t>
+          <t>4389</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E96" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-241.55</v>
       </c>
     </row>
     <row r="97">
@@ -2278,16 +2278,16 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>4124</t>
+          <t>4390</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E97" s="1" t="n">
-        <v>-133425.67</v>
+        <v>-7954.55</v>
       </c>
     </row>
     <row r="98">
@@ -2298,16 +2298,16 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>4125</t>
+          <t>4391</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E98" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-53438.85</v>
       </c>
     </row>
     <row r="99">
@@ -2318,16 +2318,16 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>4126</t>
+          <t>4392</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E99" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-133380.79</v>
       </c>
     </row>
     <row r="100">
@@ -2338,76 +2338,76 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>4127</t>
+          <t>4393</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E100" s="1" t="n">
-        <v>-7866.58</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>05/18/2026</t>
+          <t>04/20/2026</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>4131</t>
+          <t>4394</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E101" s="1" t="n">
-        <v>-1134.1</v>
+        <v>-79747.81</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>05/18/2026</t>
+          <t>04/20/2026</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>4132</t>
+          <t>4395</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E102" s="1" t="n">
-        <v>-2045.5</v>
+        <v>-7372.83</v>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>05/18/2026</t>
+          <t>04/28/2026</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>4133</t>
+          <t>4398</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Owen Pike Hauling</t>
         </is>
       </c>
       <c r="E103" s="1" t="n">
-        <v>-241.5</v>
+        <v>-1975</v>
       </c>
     </row>
     <row r="104">
@@ -2418,16 +2418,16 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>4134</t>
+          <t>4400</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E104" s="1" t="n">
-        <v>-7954.5</v>
+        <v>-1134.1</v>
       </c>
     </row>
     <row r="105">
@@ -2438,16 +2438,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>4135</t>
+          <t>4401</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E105" s="1" t="n">
-        <v>-53438.88</v>
+        <v>-2045.5</v>
       </c>
     </row>
     <row r="106">
@@ -2458,16 +2458,16 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>4136</t>
+          <t>4402</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E106" s="1" t="n">
-        <v>-133425.69</v>
+        <v>-241.5</v>
       </c>
     </row>
     <row r="107">
@@ -2478,16 +2478,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>4137</t>
+          <t>4403</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E107" s="1" t="n">
-        <v>-1284.37</v>
+        <v>-7954.5</v>
       </c>
     </row>
     <row r="108">
@@ -2498,16 +2498,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>4138</t>
+          <t>4404</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E108" s="1" t="n">
-        <v>-79747.78999999999</v>
+        <v>-53438.88</v>
       </c>
     </row>
     <row r="109">
@@ -2518,273 +2518,333 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>4139</t>
+          <t>4405</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E109" s="1" t="n">
-        <v>-7866.57</v>
+        <v>-133380.74</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>06/02/2026</t>
+          <t>05/18/2026</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>4391</t>
+          <t>4406</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E110" s="1" t="n">
-        <v>-8750</v>
+        <v>-1284.37</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>05/18/2026</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>4393</t>
+          <t>4407</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E111" s="1" t="n">
-        <v>-22140.6</v>
+        <v>-79747.78999999999</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>06/08/2026</t>
+          <t>05/18/2026</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>4396</t>
+          <t>4408</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E112" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-7372.82</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>06/11/2026</t>
+          <t>06/02/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>4399</t>
+          <t>4411</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E113" s="1" t="n">
-        <v>-3915</v>
+        <v>-8750</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>06/16/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>4402</t>
+          <t>4412</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E114" s="1" t="n">
-        <v>-17480.25</v>
+        <v>-22140.6</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>06/19/2026</t>
+          <t>06/08/2026</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>4405</t>
+          <t>4413</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E115" s="1" t="n">
-        <v>-4210</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>06/22/2026</t>
+          <t>06/11/2026</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>4408</t>
+          <t>4414</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E116" s="1" t="n">
-        <v>-15600</v>
+        <v>-3915</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>06/22/2026</t>
+          <t>06/16/2026</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>4412</t>
+          <t>4415</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E117" s="1" t="n">
-        <v>-2480</v>
+        <v>-17480.25</v>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>06/26/2026</t>
+          <t>06/19/2026</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>4418</t>
+          <t>4416</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E118" s="1" t="n">
-        <v>-8750</v>
+        <v>-4210</v>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>06/27/2026</t>
+          <t>06/22/2026</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>4421</t>
+          <t>4417</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Tri-County Tool Rental</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E119" s="1" t="n">
-        <v>-3100</v>
+        <v>-15600</v>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>06/29/2026</t>
+          <t>06/22/2026</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>4425</t>
+          <t>4418</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E120" s="1" t="n">
-        <v>-1780</v>
+        <v>-2480</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Granite Peak Properties</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="n">
+        <v>-8750</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>06/27/2026</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>4421</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Tri-County Tool Rental</t>
+        </is>
+      </c>
+      <c r="E122" s="1" t="n">
+        <v>-3100</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>06/29/2026</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>4425</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Alder &amp; Finch CPAs</t>
+        </is>
+      </c>
+      <c r="E123" s="1" t="n">
+        <v>-1780</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" t="inlineStr">
+        <is>
           <t>06/30/2026</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>4427</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>4426</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
         <is>
           <t>Moraine Cycle Components</t>
         </is>
       </c>
-      <c r="E121" s="1" t="n">
+      <c r="E124" s="1" t="n">
         <v>-11265.4</v>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
+    <row r="125">
+      <c r="A125" t="inlineStr">
         <is>
           <t>Total for 10100 Checking - First Prairie</t>
         </is>
       </c>
-      <c r="E122" s="1" t="n">
+      <c r="E125" s="1" t="n">
         <v>-3285040.78</v>
       </c>
     </row>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126">
-      <c r="A126" t="inlineStr">
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129">
+      <c r="A129" t="inlineStr">
         <is>
           <t xml:space="preserve"> Wednesday, July 15, 2026 10:50 AM GMTZ</t>
         </is>

</xml_diff>

<commit_message>
E3: self-approved payments and a round trip in Kestrel; neutral company name in the round-trip test
- Engine: Payment_approvals role and forensic.self_approved_payments, which
  reads an approval or signature log kept apart from the payment register.
  Tested on invented data.
- Engine fix: forensic.closed_value_flow named every client "Rockwood"; it
  now uses a neutral name. No result changed (a payment's outflow ends at a
  vendor node, so every leg must be in Value_flows; stated in the code).
- Kestrel: check_signatures.csv (Dana Merritt prepared and signed the three
  DM Consulting checks) and flow_of_funds.csv (Kestrel -> Gallatin Display
  Works -> Summit Loop Racing -> Kestrel, 9,800). Trial balances unchanged.
  Key lines, check_key.py 24/24, finish line 172/174, 0 unexplained.

532 tests pass; check-lessons passes. Not reviewed by a second agent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/case-studies/kestrel-valley-cycle/data/quickbooks/Bill_Payment_List.xlsx
+++ b/case-studies/kestrel-valley-cycle/data/quickbooks/Bill_Payment_List.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4268</t>
+          <t>4267</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4269</t>
+          <t>4268</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>4270</t>
+          <t>4269</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4271</t>
+          <t>4270</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4272</t>
+          <t>4271</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="E11" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="12">
@@ -578,7 +578,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4273</t>
+          <t>4272</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="E12" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +598,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4274</t>
+          <t>4273</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4275</t>
+          <t>4274</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="E14" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="15">
@@ -638,7 +638,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4276</t>
+          <t>4275</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>4281</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>4282</t>
+          <t>4281</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4283</t>
+          <t>4282</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4284</t>
+          <t>4283</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>4285</t>
+          <t>4284</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="E20" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="21">
@@ -758,7 +758,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4286</t>
+          <t>4285</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E21" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="22">
@@ -778,7 +778,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4287</t>
+          <t>4286</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4288</t>
+          <t>4287</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="E23" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="24">
@@ -818,7 +818,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4289</t>
+          <t>4288</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4293</t>
+          <t>4292</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4294</t>
+          <t>4293</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4295</t>
+          <t>4294</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4296</t>
+          <t>4295</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4297</t>
+          <t>4296</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="E29" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="30">
@@ -938,7 +938,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4298</t>
+          <t>4297</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="E30" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="31">
@@ -958,7 +958,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>4299</t>
+          <t>4298</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4300</t>
+          <t>4299</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="E32" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="33">
@@ -998,7 +998,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4301</t>
+          <t>4300</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>4303</t>
+          <t>4302</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>4308</t>
+          <t>4307</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>4309</t>
+          <t>4308</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>4310</t>
+          <t>4309</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>4311</t>
+          <t>4310</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>4312</t>
+          <t>4311</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="E39" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="40">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>4313</t>
+          <t>4312</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="E40" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="41">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>4314</t>
+          <t>4313</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>4315</t>
+          <t>4314</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="E42" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="43">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>4316</t>
+          <t>4315</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>4320</t>
+          <t>4319</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>4321</t>
+          <t>4320</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>4322</t>
+          <t>4321</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>4323</t>
+          <t>4322</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>4324</t>
+          <t>4323</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>4325</t>
+          <t>4324</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>4326</t>
+          <t>4325</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>4327</t>
+          <t>4326</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="E51" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="52">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>4328</t>
+          <t>4327</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="E52" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="53">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4329</t>
+          <t>4328</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>4330</t>
+          <t>4329</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="E54" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="55">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>4331</t>
+          <t>4330</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>4335</t>
+          <t>4334</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>4336</t>
+          <t>4335</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>4337</t>
+          <t>4336</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>4338</t>
+          <t>4337</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>4339</t>
+          <t>4338</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="E60" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="61">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>4340</t>
+          <t>4339</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="E61" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="62">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>4341</t>
+          <t>4340</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>4342</t>
+          <t>4341</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E63" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="64">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>4343</t>
+          <t>4342</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>4348</t>
+          <t>4347</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>4349</t>
+          <t>4348</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4350</t>
+          <t>4349</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>4351</t>
+          <t>4350</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>4352</t>
+          <t>4351</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="E69" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="70">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>4353</t>
+          <t>4352</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="E70" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="71">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4354</t>
+          <t>4353</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>4355</t>
+          <t>4354</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="E72" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="73">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>4356</t>
+          <t>4355</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>4359</t>
+          <t>4358</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>4361</t>
+          <t>4360</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>4362</t>
+          <t>4361</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>4363</t>
+          <t>4362</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>4364</t>
+          <t>4363</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>4365</t>
+          <t>4364</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="E79" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="80">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>4366</t>
+          <t>4365</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="E80" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="81">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>4367</t>
+          <t>4366</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>4368</t>
+          <t>4367</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="E82" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="83">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>4369</t>
+          <t>4368</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>4373</t>
+          <t>4372</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>4374</t>
+          <t>4373</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>4375</t>
+          <t>4374</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>4376</t>
+          <t>4375</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>4377</t>
+          <t>4376</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="E88" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="89">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>4378</t>
+          <t>4377</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="E89" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="90">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>4379</t>
+          <t>4378</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>4380</t>
+          <t>4379</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="E91" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="92">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>4381</t>
+          <t>4380</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>4385</t>
+          <t>4384</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>4387</t>
+          <t>4386</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>4388</t>
+          <t>4387</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>4389</t>
+          <t>4388</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>4390</t>
+          <t>4389</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>4391</t>
+          <t>4390</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="E98" s="1" t="n">
-        <v>-53438.85</v>
+        <v>-53278.49</v>
       </c>
     </row>
     <row r="99">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>4392</t>
+          <t>4391</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="E99" s="1" t="n">
-        <v>-133380.79</v>
+        <v>-132890.78</v>
       </c>
     </row>
     <row r="100">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>4393</t>
+          <t>4392</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>4394</t>
+          <t>4393</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="E101" s="1" t="n">
-        <v>-79747.81</v>
+        <v>-79507.25999999999</v>
       </c>
     </row>
     <row r="102">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>4395</t>
+          <t>4394</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>4398</t>
+          <t>4397</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2413,21 +2413,21 @@
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>05/18/2026</t>
+          <t>05/12/2026</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>4400</t>
+          <t>4399</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Gallatin Display Works</t>
         </is>
       </c>
       <c r="E104" s="1" t="n">
-        <v>-1134.1</v>
+        <v>-9800</v>
       </c>
     </row>
     <row r="105">
@@ -2438,16 +2438,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>4401</t>
+          <t>4400</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Alder &amp; Finch CPAs</t>
         </is>
       </c>
       <c r="E105" s="1" t="n">
-        <v>-2045.5</v>
+        <v>-1134.1</v>
       </c>
     </row>
     <row r="106">
@@ -2458,16 +2458,16 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>4402</t>
+          <t>4401</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Big Timber Office Supply</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E106" s="1" t="n">
-        <v>-241.5</v>
+        <v>-2045.5</v>
       </c>
     </row>
     <row r="107">
@@ -2478,16 +2478,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>4403</t>
+          <t>4402</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Big Timber Office Supply</t>
         </is>
       </c>
       <c r="E107" s="1" t="n">
-        <v>-7954.5</v>
+        <v>-241.5</v>
       </c>
     </row>
     <row r="108">
@@ -2498,16 +2498,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>4404</t>
+          <t>4403</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Kinetic Drivetrain Co.</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E108" s="1" t="n">
-        <v>-53438.88</v>
+        <v>-7954.5</v>
       </c>
     </row>
     <row r="109">
@@ -2518,16 +2518,16 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>4405</t>
+          <t>4404</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Kinetic Drivetrain Co.</t>
         </is>
       </c>
       <c r="E109" s="1" t="n">
-        <v>-133380.74</v>
+        <v>-53278.51</v>
       </c>
     </row>
     <row r="110">
@@ -2538,16 +2538,16 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>4406</t>
+          <t>4405</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E110" s="1" t="n">
-        <v>-1284.37</v>
+        <v>-132890.82</v>
       </c>
     </row>
     <row r="111">
@@ -2558,16 +2558,16 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>4407</t>
+          <t>4406</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E111" s="1" t="n">
-        <v>-79747.78999999999</v>
+        <v>-1284.37</v>
       </c>
     </row>
     <row r="112">
@@ -2578,156 +2578,156 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>4408</t>
+          <t>4407</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E112" s="1" t="n">
-        <v>-7372.82</v>
+        <v>-79507.28</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>06/02/2026</t>
+          <t>05/18/2026</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>4411</t>
+          <t>4408</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E113" s="1" t="n">
-        <v>-8750</v>
+        <v>-7372.82</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>06/02/2026</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>4412</t>
+          <t>4411</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E114" s="1" t="n">
-        <v>-22140.6</v>
+        <v>-8750</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>06/08/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>4413</t>
+          <t>4412</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Northwestern Energy</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E115" s="1" t="n">
-        <v>-1284.33</v>
+        <v>-22140.6</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>06/11/2026</t>
+          <t>06/08/2026</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>4414</t>
+          <t>4413</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Northwestern Energy</t>
         </is>
       </c>
       <c r="E116" s="1" t="n">
-        <v>-3915</v>
+        <v>-1284.33</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>06/16/2026</t>
+          <t>06/11/2026</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>4415</t>
+          <t>4414</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Summit Tire Import</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E117" s="1" t="n">
-        <v>-17480.25</v>
+        <v>-3915</v>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>06/19/2026</t>
+          <t>06/16/2026</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>4416</t>
+          <t>4415</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Big Hole Insurance</t>
+          <t>Summit Tire Import</t>
         </is>
       </c>
       <c r="E118" s="1" t="n">
-        <v>-4210</v>
+        <v>-17480.25</v>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>06/22/2026</t>
+          <t>06/19/2026</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>4417</t>
+          <t>4416</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Moraine Cycle Components</t>
+          <t>Big Hole Insurance</t>
         </is>
       </c>
       <c r="E119" s="1" t="n">
-        <v>-15600</v>
+        <v>-4210</v>
       </c>
     </row>
     <row r="120">
@@ -2738,113 +2738,133 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>4418</t>
+          <t>4417</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Velo Freight Lines</t>
+          <t>Moraine Cycle Components</t>
         </is>
       </c>
       <c r="E120" s="1" t="n">
-        <v>-2480</v>
+        <v>-15600</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>06/26/2026</t>
+          <t>06/22/2026</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>4420</t>
+          <t>4418</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Granite Peak Properties</t>
+          <t>Velo Freight Lines</t>
         </is>
       </c>
       <c r="E121" s="1" t="n">
-        <v>-8750</v>
+        <v>-2480</v>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>06/27/2026</t>
+          <t>06/26/2026</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>4421</t>
+          <t>4420</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Tri-County Tool Rental</t>
+          <t>Granite Peak Properties</t>
         </is>
       </c>
       <c r="E122" s="1" t="n">
-        <v>-3100</v>
+        <v>-8750</v>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>06/29/2026</t>
+          <t>06/27/2026</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>4425</t>
+          <t>4421</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Alder &amp; Finch CPAs</t>
+          <t>Tri-County Tool Rental</t>
         </is>
       </c>
       <c r="E123" s="1" t="n">
-        <v>-1780</v>
+        <v>-3100</v>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
+          <t>06/29/2026</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>4425</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Alder &amp; Finch CPAs</t>
+        </is>
+      </c>
+      <c r="E124" s="1" t="n">
+        <v>-1780</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" t="inlineStr">
+        <is>
           <t>06/30/2026</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
+      <c r="C125" t="inlineStr">
         <is>
           <t>4426</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="D125" t="inlineStr">
         <is>
           <t>Moraine Cycle Components</t>
         </is>
       </c>
-      <c r="E124" s="1" t="n">
+      <c r="E125" s="1" t="n">
         <v>-11265.4</v>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
+    <row r="126">
+      <c r="A126" t="inlineStr">
         <is>
           <t>Total for 10100 Checking - First Prairie</t>
         </is>
       </c>
-      <c r="E125" s="1" t="n">
+      <c r="E126" s="1" t="n">
         <v>-3285040.78</v>
       </c>
     </row>
-    <row r="126"/>
     <row r="127"/>
     <row r="128"/>
-    <row r="129">
-      <c r="A129" t="inlineStr">
+    <row r="129"/>
+    <row r="130">
+      <c r="A130" t="inlineStr">
         <is>
           <t xml:space="preserve"> Wednesday, July 15, 2026 10:50 AM GMTZ</t>
         </is>

</xml_diff>